<commit_message>
Identifie Alain McKenna et lui donne son vrai angle
A. McKenna devient Alain McKenna, du Devoir. Il n'a pas couvert l'asclépiade:
il a écrit « Des écouteurs de Québec pour oublier les AirPods » le 24 décembre
2021, sur Sounds Good, la première entreprise de Gabriel, à l'époque des trois
associés.

L'angle est donc la continuité de l'entrepreneur, pas la matière. Son brouillon
dit d'entrée que Gabriel a vendu ses parts en 2022, parce que McKenna suit
encore cette entreprise-là et le vérifierait. Il oppose ensuite les deux
projets: importer un produit existant et le vendre mieux, contre bâtir une
chaîne d'approvisionnement qui n'existe pas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_listes_medias_2026_brouillons.xlsx
+++ b/communique-dragons/Lasclay_listes_medias_2026_brouillons.xlsx
@@ -3007,7 +3007,7 @@
     <row r="31" ht="15" customHeight="1" s="26">
       <c r="A31" s="36" t="inlineStr">
         <is>
-          <t>A. McKenna</t>
+          <t>Alain McKenna</t>
         </is>
       </c>
       <c r="B31" s="36" t="inlineStr">
@@ -3020,21 +3020,33 @@
           <t>amckenna@ledevoir.com</t>
         </is>
       </c>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="37" t="n"/>
+      <c r="D31" s="36" t="inlineStr">
+        <is>
+          <t>2021-12-24</t>
+        </is>
+      </c>
+      <c r="E31" s="37" t="inlineStr">
+        <is>
+          <t>Des écouteurs de Québec pour oublier les AirPods (Sounds Good)</t>
+        </is>
+      </c>
       <c r="F31" s="36" t="inlineStr">
         <is>
-          <t>Fournie par Gabriel</t>
+          <t>Lien fourni par Gabriel</t>
         </is>
       </c>
       <c r="G31" s="40" t="inlineStr">
         <is>
-          <t>Non recoupée dans Missive</t>
+          <t>Correspondance confirmée</t>
         </is>
       </c>
       <c r="H31" s="38" t="n"/>
       <c r="I31" s="38" t="n"/>
-      <c r="J31" s="39" t="n"/>
+      <c r="J31" s="39" t="inlineStr">
+        <is>
+          <t>A couvert Sounds Good, la première entreprise de Gabriel, à l'époque des trois associés. Gabriel a vendu ses parts en 2022 : le dire d'entrée, McKenna suit encore Sounds Good.</t>
+        </is>
+      </c>
       <c r="K31" s="25" t="inlineStr">
         <is>
           <t>A</t>
@@ -3042,25 +3054,29 @@
       </c>
       <c r="L31" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de [année] sur l'asclepiade</t>
+          <t>Suite a votre article de 2021 sur les ecouteurs de Quebec</t>
         </is>
       </c>
       <c r="M31" s="25" t="inlineStr">
         <is>
-          <t>Bonjour,</t>
+          <t>Bonjour Alain,</t>
         </is>
       </c>
       <c r="N31" s="46" t="inlineStr">
         <is>
-          <t>Bonjour [Prénom],
-Lasclay est une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile.
-Le 17 septembre, on est dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et
-CBC Gem.
-L'histoire d'affaires, si elle vous intéresse : on a rapatrié notre production en 2021 faute
-de sous-traitant prêt à toucher à la fibre, puis on a confié l'assemblage textile à
-l'externe en 2025 pour rendre un manteau accessible à 300 $. Les deux décisions se
-défendent, et elles se contredisent en apparence.
-Je ne peux pas dire comment la rencontre s'est terminée avant la diffusion.</t>
+          <t>Bonjour Alain,
+Vous aviez écrit « Des écouteurs de Québec pour oublier les AirPods » le 24 décembre 2021,
+sur Sounds Good et ses écouteurs à 99,99 $. J'étais un des trois.
+J'ai vendu mes parts en 2022 pour me consacrer à l'autre entreprise que j'avais démarrée
+entretemps : Lasclay, qui transforme la soie d'asclépiade en isolant textile. Sounds Good
+continue sans moi.
+Le 17 septembre, Lasclay est dans le premier épisode de la 21e saison de Dragons' Den, sur
+CBC et CBC Gem. Je ne peux pas dire comment ça s'est terminé avant la diffusion.
+Ce qui pourrait vous intéresser : c'est le contraire exact de Sounds Good. Là-bas, on
+importait un produit existant et on le vendait mieux. Ici, il n'y a aucune chaîne
+d'approvisionnement, alors on a bâti nos propres procédés en 2021, puis on a sorti
+l'assemblage textile du Québec en 2025 pour rendre un manteau accessible à 300 $. Les deux
+décisions se défendent et elles se contredisent en apparence.</t>
         </is>
       </c>
     </row>

</xml_diff>